<commit_message>
Keep Excel schedule dates consistent across browser timezones
</commit_message>
<xml_diff>
--- a/assets/business-test-data/all_tables.xlsx
+++ b/assets/business-test-data/all_tables.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stores" sheetId="1" r:id="Rf9887fafc1184a68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="role_permissions" sheetId="2" r:id="R51097ebab4d14a47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="staff" sheetId="3" r:id="Rac8e228c07ef4473"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="devices" sheetId="4" r:id="R3c274ffd7dfa41a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories_100" sheetId="5" r:id="Re6f3829c7a374a24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="brands" sheetId="6" r:id="R38dfd33ea7c340b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="suppliers" sheetId="7" r:id="Rc319647d8e664056"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="storage_locations" sheetId="8" r:id="R950b527252f14d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="products_100" sheetId="9" r:id="Rf3ce56adadf34ea3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_products_100" sheetId="10" r:id="Re0c451766da14275"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_extras" sheetId="11" r:id="Rf8d3570b89e04b9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="supplier_purchases" sheetId="12" r:id="Re4843ec61ee642e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stock_movements" sheetId="13" r:id="Rc14ddbd1994947b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inventory_counts" sheetId="14" r:id="Ra8f92c1130204e73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="schedules" sheetId="15" r:id="Rd0f52b356c3f46c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="timesheets" sheetId="16" r:id="Ra2c8e01abc2c4c85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sales" sheetId="17" r:id="Rf265bae22fb74a58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="login_events" sheetId="18" r:id="Rcf4a3581a7984508"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_stores" sheetId="19" r:id="Re19157407ae04d8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stores" sheetId="1" r:id="R3451f0fc465548f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="role_permissions" sheetId="2" r:id="Rc90fae817c27417c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="staff" sheetId="3" r:id="Ra299991c6d0e479a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="devices" sheetId="4" r:id="Rf72e791bdca449d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories_100" sheetId="5" r:id="R5ebdb9a6a4814e2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="brands" sheetId="6" r:id="R8995c8904a57460c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="suppliers" sheetId="7" r:id="Rba92e87735f44f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="storage_locations" sheetId="8" r:id="R7b6ae9bb5def4413"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="products_100" sheetId="9" r:id="R434f4e22c0734d57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_products_100" sheetId="10" r:id="R00ca5308e6494fca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_extras" sheetId="11" r:id="Reb076b2bc02d41eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="supplier_purchases" sheetId="12" r:id="R39d269db757145cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stock_movements" sheetId="13" r:id="Ra673e325e6aa49a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inventory_counts" sheetId="14" r:id="R9facafab769547d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="schedules" sheetId="15" r:id="R702c906cd1f447e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="timesheets" sheetId="16" r:id="R979f42c95acd45aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sales" sheetId="17" r:id="Rf7615217799f46fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="login_events" sheetId="18" r:id="R9e8fbb5eb1d64eab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_stores" sheetId="19" r:id="Rca13fcb8d4c74ac8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31,6 +31,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd&quot;T&quot;hh:mm:ss&quot;Z&quot;"/>
+  </x:numFmts>
   <x:fonts count="1">
     <x:font>
       <x:sz val="11"/>
@@ -62,7 +65,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="3">
+  <x:cellXfs count="4">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
@@ -72,6 +75,7 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -8532,8 +8536,8 @@
     <x:col min="1" max="1" width="21" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="29" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="29" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -8561,10 +8565,10 @@
         <x:v>STAFF001</x:v>
       </x:c>
       <x:c r="C2" t="str"/>
-      <x:c r="D2" t="d">
+      <x:c r="D2" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E2" t="d">
+      <x:c r="E2" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8576,10 +8580,10 @@
         <x:v>STAFF002</x:v>
       </x:c>
       <x:c r="C3" t="str"/>
-      <x:c r="D3" t="d">
+      <x:c r="D3" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E3" t="d">
+      <x:c r="E3" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8591,10 +8595,10 @@
         <x:v>STAFF003</x:v>
       </x:c>
       <x:c r="C4" t="str"/>
-      <x:c r="D4" t="d">
+      <x:c r="D4" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E4" t="d">
+      <x:c r="E4" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8606,10 +8610,10 @@
         <x:v>STAFF004</x:v>
       </x:c>
       <x:c r="C5" t="str"/>
-      <x:c r="D5" t="d">
+      <x:c r="D5" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E5" t="d">
+      <x:c r="E5" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8621,10 +8625,10 @@
         <x:v>STAFF005</x:v>
       </x:c>
       <x:c r="C6" t="str"/>
-      <x:c r="D6" t="d">
+      <x:c r="D6" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E6" t="d">
+      <x:c r="E6" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8636,10 +8640,10 @@
         <x:v>STAFF006</x:v>
       </x:c>
       <x:c r="C7" t="str"/>
-      <x:c r="D7" t="d">
+      <x:c r="D7" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E7" t="d">
+      <x:c r="E7" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8651,10 +8655,10 @@
         <x:v>STAFF007</x:v>
       </x:c>
       <x:c r="C8" t="str"/>
-      <x:c r="D8" t="d">
+      <x:c r="D8" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E8" t="d">
+      <x:c r="E8" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8666,10 +8670,10 @@
         <x:v>STAFF008</x:v>
       </x:c>
       <x:c r="C9" t="str"/>
-      <x:c r="D9" t="d">
+      <x:c r="D9" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E9" t="d">
+      <x:c r="E9" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8681,10 +8685,10 @@
         <x:v>STAFF009</x:v>
       </x:c>
       <x:c r="C10" t="str"/>
-      <x:c r="D10" t="d">
+      <x:c r="D10" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E10" t="d">
+      <x:c r="E10" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8696,10 +8700,10 @@
         <x:v>STAFF010</x:v>
       </x:c>
       <x:c r="C11" t="str"/>
-      <x:c r="D11" t="d">
+      <x:c r="D11" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E11" t="d">
+      <x:c r="E11" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8715,8 +8719,8 @@
     <x:col min="1" max="1" width="21" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="29" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="29" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -8748,10 +8752,10 @@
         <x:v>STAFF001</x:v>
       </x:c>
       <x:c r="C2" t="str"/>
-      <x:c r="D2" t="d">
+      <x:c r="D2" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E2" t="d">
+      <x:c r="E2" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F2" t="n">
@@ -8766,10 +8770,10 @@
         <x:v>STAFF002</x:v>
       </x:c>
       <x:c r="C3" t="str"/>
-      <x:c r="D3" t="d">
+      <x:c r="D3" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E3" t="d">
+      <x:c r="E3" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F3" t="n">
@@ -8784,10 +8788,10 @@
         <x:v>STAFF003</x:v>
       </x:c>
       <x:c r="C4" t="str"/>
-      <x:c r="D4" t="d">
+      <x:c r="D4" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E4" t="d">
+      <x:c r="E4" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F4" t="n">
@@ -8802,10 +8806,10 @@
         <x:v>STAFF004</x:v>
       </x:c>
       <x:c r="C5" t="str"/>
-      <x:c r="D5" t="d">
+      <x:c r="D5" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E5" t="d">
+      <x:c r="E5" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F5" t="n">
@@ -8820,10 +8824,10 @@
         <x:v>STAFF005</x:v>
       </x:c>
       <x:c r="C6" t="str"/>
-      <x:c r="D6" t="d">
+      <x:c r="D6" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E6" t="d">
+      <x:c r="E6" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F6" t="n">
@@ -8838,10 +8842,10 @@
         <x:v>STAFF006</x:v>
       </x:c>
       <x:c r="C7" t="str"/>
-      <x:c r="D7" t="d">
+      <x:c r="D7" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E7" t="d">
+      <x:c r="E7" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F7" t="n">
@@ -8856,10 +8860,10 @@
         <x:v>STAFF007</x:v>
       </x:c>
       <x:c r="C8" t="str"/>
-      <x:c r="D8" t="d">
+      <x:c r="D8" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E8" t="d">
+      <x:c r="E8" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F8" t="n">
@@ -8874,10 +8878,10 @@
         <x:v>STAFF008</x:v>
       </x:c>
       <x:c r="C9" t="str"/>
-      <x:c r="D9" t="d">
+      <x:c r="D9" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E9" t="d">
+      <x:c r="E9" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F9" t="n">
@@ -8892,10 +8896,10 @@
         <x:v>STAFF009</x:v>
       </x:c>
       <x:c r="C10" t="str"/>
-      <x:c r="D10" t="d">
+      <x:c r="D10" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E10" t="d">
+      <x:c r="E10" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F10" t="n">
@@ -8910,10 +8914,10 @@
         <x:v>STAFF010</x:v>
       </x:c>
       <x:c r="C11" t="str"/>
-      <x:c r="D11" t="d">
+      <x:c r="D11" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E11" t="d">
+      <x:c r="E11" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F11" t="n">
@@ -8928,10 +8932,10 @@
         <x:v>STAFF001</x:v>
       </x:c>
       <x:c r="C12" t="str"/>
-      <x:c r="D12" t="d">
+      <x:c r="D12" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E12" t="d">
+      <x:c r="E12" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F12" t="n">
@@ -8946,10 +8950,10 @@
         <x:v>STAFF002</x:v>
       </x:c>
       <x:c r="C13" t="str"/>
-      <x:c r="D13" t="d">
+      <x:c r="D13" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E13" t="d">
+      <x:c r="E13" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F13" t="n">
@@ -8964,10 +8968,10 @@
         <x:v>STAFF003</x:v>
       </x:c>
       <x:c r="C14" t="str"/>
-      <x:c r="D14" t="d">
+      <x:c r="D14" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E14" t="d">
+      <x:c r="E14" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F14" t="n">
@@ -8982,10 +8986,10 @@
         <x:v>STAFF004</x:v>
       </x:c>
       <x:c r="C15" t="str"/>
-      <x:c r="D15" t="d">
+      <x:c r="D15" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E15" t="d">
+      <x:c r="E15" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F15" t="n">
@@ -9000,10 +9004,10 @@
         <x:v>STAFF005</x:v>
       </x:c>
       <x:c r="C16" t="str"/>
-      <x:c r="D16" t="d">
+      <x:c r="D16" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E16" t="d">
+      <x:c r="E16" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F16" t="n">
@@ -9018,10 +9022,10 @@
         <x:v>STAFF006</x:v>
       </x:c>
       <x:c r="C17" t="str"/>
-      <x:c r="D17" t="d">
+      <x:c r="D17" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E17" t="d">
+      <x:c r="E17" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F17" t="n">
@@ -9036,10 +9040,10 @@
         <x:v>STAFF007</x:v>
       </x:c>
       <x:c r="C18" t="str"/>
-      <x:c r="D18" t="d">
+      <x:c r="D18" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E18" t="d">
+      <x:c r="E18" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F18" t="n">
@@ -9054,10 +9058,10 @@
         <x:v>STAFF008</x:v>
       </x:c>
       <x:c r="C19" t="str"/>
-      <x:c r="D19" t="d">
+      <x:c r="D19" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E19" t="d">
+      <x:c r="E19" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F19" t="n">
@@ -9072,10 +9076,10 @@
         <x:v>STAFF009</x:v>
       </x:c>
       <x:c r="C20" t="str"/>
-      <x:c r="D20" t="d">
+      <x:c r="D20" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E20" t="d">
+      <x:c r="E20" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F20" t="n">
@@ -9090,10 +9094,10 @@
         <x:v>STAFF010</x:v>
       </x:c>
       <x:c r="C21" t="str"/>
-      <x:c r="D21" t="d">
+      <x:c r="D21" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E21" t="d">
+      <x:c r="E21" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F21" t="n">
@@ -12670,7 +12674,7 @@
     <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="29" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="21" hidden="0" customWidth="1"/>
   </x:cols>
@@ -12711,7 +12715,7 @@
       <x:c r="D2" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E2" t="d">
+      <x:c r="E2" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F2" t="str">
@@ -12734,7 +12738,7 @@
       <x:c r="D3" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E3" t="d">
+      <x:c r="E3" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F3" t="str">
@@ -12757,7 +12761,7 @@
       <x:c r="D4" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E4" t="d">
+      <x:c r="E4" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F4" t="str">
@@ -12780,7 +12784,7 @@
       <x:c r="D5" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E5" t="d">
+      <x:c r="E5" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F5" t="str">
@@ -12803,7 +12807,7 @@
       <x:c r="D6" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E6" t="d">
+      <x:c r="E6" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F6" t="str">
@@ -12826,7 +12830,7 @@
       <x:c r="D7" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E7" t="d">
+      <x:c r="E7" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F7" t="str">
@@ -12849,7 +12853,7 @@
       <x:c r="D8" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E8" t="d">
+      <x:c r="E8" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F8" t="str">
@@ -12872,7 +12876,7 @@
       <x:c r="D9" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E9" t="d">
+      <x:c r="E9" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F9" t="str">
@@ -12895,7 +12899,7 @@
       <x:c r="D10" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E10" t="d">
+      <x:c r="E10" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F10" t="str">
@@ -12918,7 +12922,7 @@
       <x:c r="D11" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E11" t="d">
+      <x:c r="E11" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F11" t="str">
@@ -12941,7 +12945,7 @@
       <x:c r="D12" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E12" t="d">
+      <x:c r="E12" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F12" t="str">
@@ -12964,7 +12968,7 @@
       <x:c r="D13" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E13" t="d">
+      <x:c r="E13" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F13" t="str">
@@ -12987,7 +12991,7 @@
       <x:c r="D14" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E14" t="d">
+      <x:c r="E14" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F14" t="str">
@@ -13010,7 +13014,7 @@
       <x:c r="D15" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E15" t="d">
+      <x:c r="E15" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F15" t="str">
@@ -13033,7 +13037,7 @@
       <x:c r="D16" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E16" t="d">
+      <x:c r="E16" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F16" t="str">
@@ -13056,7 +13060,7 @@
       <x:c r="D17" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E17" t="d">
+      <x:c r="E17" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F17" t="str">
@@ -13079,7 +13083,7 @@
       <x:c r="D18" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E18" t="d">
+      <x:c r="E18" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F18" t="str">
@@ -13102,7 +13106,7 @@
       <x:c r="D19" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E19" t="d">
+      <x:c r="E19" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F19" t="str">
@@ -13125,7 +13129,7 @@
       <x:c r="D20" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E20" t="d">
+      <x:c r="E20" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F20" t="str">
@@ -13148,7 +13152,7 @@
       <x:c r="D21" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E21" t="d">
+      <x:c r="E21" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F21" t="str">
@@ -13171,7 +13175,7 @@
       <x:c r="D22" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E22" t="d">
+      <x:c r="E22" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F22" t="str">
@@ -13194,7 +13198,7 @@
       <x:c r="D23" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E23" t="d">
+      <x:c r="E23" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F23" t="str">
@@ -13217,7 +13221,7 @@
       <x:c r="D24" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E24" t="d">
+      <x:c r="E24" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F24" t="str">
@@ -13240,7 +13244,7 @@
       <x:c r="D25" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E25" t="d">
+      <x:c r="E25" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F25" t="str">
@@ -13263,7 +13267,7 @@
       <x:c r="D26" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E26" t="d">
+      <x:c r="E26" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F26" t="str">
@@ -13286,7 +13290,7 @@
       <x:c r="D27" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E27" t="d">
+      <x:c r="E27" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F27" t="str">
@@ -13309,7 +13313,7 @@
       <x:c r="D28" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E28" t="d">
+      <x:c r="E28" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F28" t="str">
@@ -13332,7 +13336,7 @@
       <x:c r="D29" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E29" t="d">
+      <x:c r="E29" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F29" t="str">
@@ -13355,7 +13359,7 @@
       <x:c r="D30" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E30" t="d">
+      <x:c r="E30" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F30" t="str">
@@ -13378,7 +13382,7 @@
       <x:c r="D31" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E31" t="d">
+      <x:c r="E31" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F31" t="str">
@@ -13401,7 +13405,7 @@
       <x:c r="D32" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E32" t="d">
+      <x:c r="E32" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F32" t="str">
@@ -13424,7 +13428,7 @@
       <x:c r="D33" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E33" t="d">
+      <x:c r="E33" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F33" t="str">
@@ -13447,7 +13451,7 @@
       <x:c r="D34" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E34" t="d">
+      <x:c r="E34" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F34" t="str">
@@ -13470,7 +13474,7 @@
       <x:c r="D35" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E35" t="d">
+      <x:c r="E35" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F35" t="str">
@@ -13493,7 +13497,7 @@
       <x:c r="D36" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E36" t="d">
+      <x:c r="E36" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F36" t="str">
@@ -13516,7 +13520,7 @@
       <x:c r="D37" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E37" t="d">
+      <x:c r="E37" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F37" t="str">
@@ -13539,7 +13543,7 @@
       <x:c r="D38" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E38" t="d">
+      <x:c r="E38" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F38" t="str">
@@ -13562,7 +13566,7 @@
       <x:c r="D39" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E39" t="d">
+      <x:c r="E39" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F39" t="str">
@@ -13585,7 +13589,7 @@
       <x:c r="D40" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E40" t="d">
+      <x:c r="E40" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F40" t="str">
@@ -13608,7 +13612,7 @@
       <x:c r="D41" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E41" t="d">
+      <x:c r="E41" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F41" t="str">

</xml_diff>

<commit_message>
Correct Excel date imports and publish formatted sample workbook [skip render]
</commit_message>
<xml_diff>
--- a/assets/business-test-data/all_tables.xlsx
+++ b/assets/business-test-data/all_tables.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stores" sheetId="1" r:id="Rf9887fafc1184a68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="role_permissions" sheetId="2" r:id="R51097ebab4d14a47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="staff" sheetId="3" r:id="Rac8e228c07ef4473"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="devices" sheetId="4" r:id="R3c274ffd7dfa41a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories_100" sheetId="5" r:id="Re6f3829c7a374a24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="brands" sheetId="6" r:id="R38dfd33ea7c340b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="suppliers" sheetId="7" r:id="Rc319647d8e664056"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="storage_locations" sheetId="8" r:id="R950b527252f14d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="products_100" sheetId="9" r:id="Rf3ce56adadf34ea3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_products_100" sheetId="10" r:id="Re0c451766da14275"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_extras" sheetId="11" r:id="Rf8d3570b89e04b9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="supplier_purchases" sheetId="12" r:id="Re4843ec61ee642e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stock_movements" sheetId="13" r:id="Rc14ddbd1994947b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inventory_counts" sheetId="14" r:id="Ra8f92c1130204e73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="schedules" sheetId="15" r:id="Rd0f52b356c3f46c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="timesheets" sheetId="16" r:id="Ra2c8e01abc2c4c85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sales" sheetId="17" r:id="Rf265bae22fb74a58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="login_events" sheetId="18" r:id="Rcf4a3581a7984508"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_stores" sheetId="19" r:id="Re19157407ae04d8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stores" sheetId="1" r:id="R3451f0fc465548f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="role_permissions" sheetId="2" r:id="Rc90fae817c27417c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="staff" sheetId="3" r:id="Ra299991c6d0e479a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="devices" sheetId="4" r:id="Rf72e791bdca449d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories_100" sheetId="5" r:id="R5ebdb9a6a4814e2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="brands" sheetId="6" r:id="R8995c8904a57460c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="suppliers" sheetId="7" r:id="Rba92e87735f44f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="storage_locations" sheetId="8" r:id="R7b6ae9bb5def4413"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="products_100" sheetId="9" r:id="R434f4e22c0734d57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_products_100" sheetId="10" r:id="R00ca5308e6494fca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_extras" sheetId="11" r:id="Reb076b2bc02d41eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="supplier_purchases" sheetId="12" r:id="R39d269db757145cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stock_movements" sheetId="13" r:id="Ra673e325e6aa49a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inventory_counts" sheetId="14" r:id="R9facafab769547d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="schedules" sheetId="15" r:id="R702c906cd1f447e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="timesheets" sheetId="16" r:id="R979f42c95acd45aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sales" sheetId="17" r:id="Rf7615217799f46fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="login_events" sheetId="18" r:id="R9e8fbb5eb1d64eab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant_stores" sheetId="19" r:id="Rca13fcb8d4c74ac8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31,6 +31,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd&quot;T&quot;hh:mm:ss&quot;Z&quot;"/>
+  </x:numFmts>
   <x:fonts count="1">
     <x:font>
       <x:sz val="11"/>
@@ -62,7 +65,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="3">
+  <x:cellXfs count="4">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
@@ -72,6 +75,7 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -8532,8 +8536,8 @@
     <x:col min="1" max="1" width="21" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="29" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="29" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -8561,10 +8565,10 @@
         <x:v>STAFF001</x:v>
       </x:c>
       <x:c r="C2" t="str"/>
-      <x:c r="D2" t="d">
+      <x:c r="D2" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E2" t="d">
+      <x:c r="E2" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8576,10 +8580,10 @@
         <x:v>STAFF002</x:v>
       </x:c>
       <x:c r="C3" t="str"/>
-      <x:c r="D3" t="d">
+      <x:c r="D3" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E3" t="d">
+      <x:c r="E3" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8591,10 +8595,10 @@
         <x:v>STAFF003</x:v>
       </x:c>
       <x:c r="C4" t="str"/>
-      <x:c r="D4" t="d">
+      <x:c r="D4" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E4" t="d">
+      <x:c r="E4" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8606,10 +8610,10 @@
         <x:v>STAFF004</x:v>
       </x:c>
       <x:c r="C5" t="str"/>
-      <x:c r="D5" t="d">
+      <x:c r="D5" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E5" t="d">
+      <x:c r="E5" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8621,10 +8625,10 @@
         <x:v>STAFF005</x:v>
       </x:c>
       <x:c r="C6" t="str"/>
-      <x:c r="D6" t="d">
+      <x:c r="D6" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E6" t="d">
+      <x:c r="E6" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8636,10 +8640,10 @@
         <x:v>STAFF006</x:v>
       </x:c>
       <x:c r="C7" t="str"/>
-      <x:c r="D7" t="d">
+      <x:c r="D7" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E7" t="d">
+      <x:c r="E7" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8651,10 +8655,10 @@
         <x:v>STAFF007</x:v>
       </x:c>
       <x:c r="C8" t="str"/>
-      <x:c r="D8" t="d">
+      <x:c r="D8" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E8" t="d">
+      <x:c r="E8" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8666,10 +8670,10 @@
         <x:v>STAFF008</x:v>
       </x:c>
       <x:c r="C9" t="str"/>
-      <x:c r="D9" t="d">
+      <x:c r="D9" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E9" t="d">
+      <x:c r="E9" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8681,10 +8685,10 @@
         <x:v>STAFF009</x:v>
       </x:c>
       <x:c r="C10" t="str"/>
-      <x:c r="D10" t="d">
+      <x:c r="D10" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E10" t="d">
+      <x:c r="E10" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8696,10 +8700,10 @@
         <x:v>STAFF010</x:v>
       </x:c>
       <x:c r="C11" t="str"/>
-      <x:c r="D11" t="d">
+      <x:c r="D11" s="3" t="d">
         <x:v>2026-10-26T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E11" t="d">
+      <x:c r="E11" s="3" t="d">
         <x:v>2026-10-26T21:00:00.000Z</x:v>
       </x:c>
     </x:row>
@@ -8715,8 +8719,8 @@
     <x:col min="1" max="1" width="21" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="29" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="29" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -8748,10 +8752,10 @@
         <x:v>STAFF001</x:v>
       </x:c>
       <x:c r="C2" t="str"/>
-      <x:c r="D2" t="d">
+      <x:c r="D2" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E2" t="d">
+      <x:c r="E2" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F2" t="n">
@@ -8766,10 +8770,10 @@
         <x:v>STAFF002</x:v>
       </x:c>
       <x:c r="C3" t="str"/>
-      <x:c r="D3" t="d">
+      <x:c r="D3" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E3" t="d">
+      <x:c r="E3" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F3" t="n">
@@ -8784,10 +8788,10 @@
         <x:v>STAFF003</x:v>
       </x:c>
       <x:c r="C4" t="str"/>
-      <x:c r="D4" t="d">
+      <x:c r="D4" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E4" t="d">
+      <x:c r="E4" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F4" t="n">
@@ -8802,10 +8806,10 @@
         <x:v>STAFF004</x:v>
       </x:c>
       <x:c r="C5" t="str"/>
-      <x:c r="D5" t="d">
+      <x:c r="D5" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E5" t="d">
+      <x:c r="E5" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F5" t="n">
@@ -8820,10 +8824,10 @@
         <x:v>STAFF005</x:v>
       </x:c>
       <x:c r="C6" t="str"/>
-      <x:c r="D6" t="d">
+      <x:c r="D6" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E6" t="d">
+      <x:c r="E6" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F6" t="n">
@@ -8838,10 +8842,10 @@
         <x:v>STAFF006</x:v>
       </x:c>
       <x:c r="C7" t="str"/>
-      <x:c r="D7" t="d">
+      <x:c r="D7" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E7" t="d">
+      <x:c r="E7" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F7" t="n">
@@ -8856,10 +8860,10 @@
         <x:v>STAFF007</x:v>
       </x:c>
       <x:c r="C8" t="str"/>
-      <x:c r="D8" t="d">
+      <x:c r="D8" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E8" t="d">
+      <x:c r="E8" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F8" t="n">
@@ -8874,10 +8878,10 @@
         <x:v>STAFF008</x:v>
       </x:c>
       <x:c r="C9" t="str"/>
-      <x:c r="D9" t="d">
+      <x:c r="D9" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E9" t="d">
+      <x:c r="E9" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F9" t="n">
@@ -8892,10 +8896,10 @@
         <x:v>STAFF009</x:v>
       </x:c>
       <x:c r="C10" t="str"/>
-      <x:c r="D10" t="d">
+      <x:c r="D10" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E10" t="d">
+      <x:c r="E10" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F10" t="n">
@@ -8910,10 +8914,10 @@
         <x:v>STAFF010</x:v>
       </x:c>
       <x:c r="C11" t="str"/>
-      <x:c r="D11" t="d">
+      <x:c r="D11" s="3" t="d">
         <x:v>2026-10-19T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E11" t="d">
+      <x:c r="E11" s="3" t="d">
         <x:v>2026-10-19T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F11" t="n">
@@ -8928,10 +8932,10 @@
         <x:v>STAFF001</x:v>
       </x:c>
       <x:c r="C12" t="str"/>
-      <x:c r="D12" t="d">
+      <x:c r="D12" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E12" t="d">
+      <x:c r="E12" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F12" t="n">
@@ -8946,10 +8950,10 @@
         <x:v>STAFF002</x:v>
       </x:c>
       <x:c r="C13" t="str"/>
-      <x:c r="D13" t="d">
+      <x:c r="D13" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E13" t="d">
+      <x:c r="E13" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F13" t="n">
@@ -8964,10 +8968,10 @@
         <x:v>STAFF003</x:v>
       </x:c>
       <x:c r="C14" t="str"/>
-      <x:c r="D14" t="d">
+      <x:c r="D14" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E14" t="d">
+      <x:c r="E14" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F14" t="n">
@@ -8982,10 +8986,10 @@
         <x:v>STAFF004</x:v>
       </x:c>
       <x:c r="C15" t="str"/>
-      <x:c r="D15" t="d">
+      <x:c r="D15" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E15" t="d">
+      <x:c r="E15" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F15" t="n">
@@ -9000,10 +9004,10 @@
         <x:v>STAFF005</x:v>
       </x:c>
       <x:c r="C16" t="str"/>
-      <x:c r="D16" t="d">
+      <x:c r="D16" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E16" t="d">
+      <x:c r="E16" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F16" t="n">
@@ -9018,10 +9022,10 @@
         <x:v>STAFF006</x:v>
       </x:c>
       <x:c r="C17" t="str"/>
-      <x:c r="D17" t="d">
+      <x:c r="D17" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E17" t="d">
+      <x:c r="E17" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F17" t="n">
@@ -9036,10 +9040,10 @@
         <x:v>STAFF007</x:v>
       </x:c>
       <x:c r="C18" t="str"/>
-      <x:c r="D18" t="d">
+      <x:c r="D18" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E18" t="d">
+      <x:c r="E18" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F18" t="n">
@@ -9054,10 +9058,10 @@
         <x:v>STAFF008</x:v>
       </x:c>
       <x:c r="C19" t="str"/>
-      <x:c r="D19" t="d">
+      <x:c r="D19" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E19" t="d">
+      <x:c r="E19" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F19" t="n">
@@ -9072,10 +9076,10 @@
         <x:v>STAFF009</x:v>
       </x:c>
       <x:c r="C20" t="str"/>
-      <x:c r="D20" t="d">
+      <x:c r="D20" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E20" t="d">
+      <x:c r="E20" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F20" t="n">
@@ -9090,10 +9094,10 @@
         <x:v>STAFF010</x:v>
       </x:c>
       <x:c r="C21" t="str"/>
-      <x:c r="D21" t="d">
+      <x:c r="D21" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
-      <x:c r="E21" t="d">
+      <x:c r="E21" s="3" t="d">
         <x:v>2026-10-20T21:00:00.000Z</x:v>
       </x:c>
       <x:c r="F21" t="n">
@@ -12670,7 +12674,7 @@
     <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="29" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="21" hidden="0" customWidth="1"/>
   </x:cols>
@@ -12711,7 +12715,7 @@
       <x:c r="D2" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E2" t="d">
+      <x:c r="E2" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F2" t="str">
@@ -12734,7 +12738,7 @@
       <x:c r="D3" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E3" t="d">
+      <x:c r="E3" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F3" t="str">
@@ -12757,7 +12761,7 @@
       <x:c r="D4" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E4" t="d">
+      <x:c r="E4" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F4" t="str">
@@ -12780,7 +12784,7 @@
       <x:c r="D5" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E5" t="d">
+      <x:c r="E5" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F5" t="str">
@@ -12803,7 +12807,7 @@
       <x:c r="D6" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E6" t="d">
+      <x:c r="E6" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F6" t="str">
@@ -12826,7 +12830,7 @@
       <x:c r="D7" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E7" t="d">
+      <x:c r="E7" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F7" t="str">
@@ -12849,7 +12853,7 @@
       <x:c r="D8" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E8" t="d">
+      <x:c r="E8" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F8" t="str">
@@ -12872,7 +12876,7 @@
       <x:c r="D9" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E9" t="d">
+      <x:c r="E9" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F9" t="str">
@@ -12895,7 +12899,7 @@
       <x:c r="D10" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E10" t="d">
+      <x:c r="E10" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F10" t="str">
@@ -12918,7 +12922,7 @@
       <x:c r="D11" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E11" t="d">
+      <x:c r="E11" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F11" t="str">
@@ -12941,7 +12945,7 @@
       <x:c r="D12" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E12" t="d">
+      <x:c r="E12" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F12" t="str">
@@ -12964,7 +12968,7 @@
       <x:c r="D13" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E13" t="d">
+      <x:c r="E13" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F13" t="str">
@@ -12987,7 +12991,7 @@
       <x:c r="D14" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E14" t="d">
+      <x:c r="E14" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F14" t="str">
@@ -13010,7 +13014,7 @@
       <x:c r="D15" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E15" t="d">
+      <x:c r="E15" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F15" t="str">
@@ -13033,7 +13037,7 @@
       <x:c r="D16" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E16" t="d">
+      <x:c r="E16" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F16" t="str">
@@ -13056,7 +13060,7 @@
       <x:c r="D17" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E17" t="d">
+      <x:c r="E17" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F17" t="str">
@@ -13079,7 +13083,7 @@
       <x:c r="D18" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E18" t="d">
+      <x:c r="E18" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F18" t="str">
@@ -13102,7 +13106,7 @@
       <x:c r="D19" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E19" t="d">
+      <x:c r="E19" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F19" t="str">
@@ -13125,7 +13129,7 @@
       <x:c r="D20" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E20" t="d">
+      <x:c r="E20" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F20" t="str">
@@ -13148,7 +13152,7 @@
       <x:c r="D21" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E21" t="d">
+      <x:c r="E21" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F21" t="str">
@@ -13171,7 +13175,7 @@
       <x:c r="D22" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E22" t="d">
+      <x:c r="E22" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F22" t="str">
@@ -13194,7 +13198,7 @@
       <x:c r="D23" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E23" t="d">
+      <x:c r="E23" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F23" t="str">
@@ -13217,7 +13221,7 @@
       <x:c r="D24" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E24" t="d">
+      <x:c r="E24" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F24" t="str">
@@ -13240,7 +13244,7 @@
       <x:c r="D25" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E25" t="d">
+      <x:c r="E25" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F25" t="str">
@@ -13263,7 +13267,7 @@
       <x:c r="D26" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E26" t="d">
+      <x:c r="E26" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F26" t="str">
@@ -13286,7 +13290,7 @@
       <x:c r="D27" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E27" t="d">
+      <x:c r="E27" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F27" t="str">
@@ -13309,7 +13313,7 @@
       <x:c r="D28" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E28" t="d">
+      <x:c r="E28" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F28" t="str">
@@ -13332,7 +13336,7 @@
       <x:c r="D29" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E29" t="d">
+      <x:c r="E29" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F29" t="str">
@@ -13355,7 +13359,7 @@
       <x:c r="D30" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E30" t="d">
+      <x:c r="E30" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F30" t="str">
@@ -13378,7 +13382,7 @@
       <x:c r="D31" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E31" t="d">
+      <x:c r="E31" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F31" t="str">
@@ -13401,7 +13405,7 @@
       <x:c r="D32" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E32" t="d">
+      <x:c r="E32" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F32" t="str">
@@ -13424,7 +13428,7 @@
       <x:c r="D33" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E33" t="d">
+      <x:c r="E33" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F33" t="str">
@@ -13447,7 +13451,7 @@
       <x:c r="D34" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E34" t="d">
+      <x:c r="E34" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F34" t="str">
@@ -13470,7 +13474,7 @@
       <x:c r="D35" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E35" t="d">
+      <x:c r="E35" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F35" t="str">
@@ -13493,7 +13497,7 @@
       <x:c r="D36" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E36" t="d">
+      <x:c r="E36" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F36" t="str">
@@ -13516,7 +13520,7 @@
       <x:c r="D37" t="str">
         <x:v>DEV001</x:v>
       </x:c>
-      <x:c r="E37" t="d">
+      <x:c r="E37" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F37" t="str">
@@ -13539,7 +13543,7 @@
       <x:c r="D38" t="str">
         <x:v>DEV002</x:v>
       </x:c>
-      <x:c r="E38" t="d">
+      <x:c r="E38" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F38" t="str">
@@ -13562,7 +13566,7 @@
       <x:c r="D39" t="str">
         <x:v>DEV003</x:v>
       </x:c>
-      <x:c r="E39" t="d">
+      <x:c r="E39" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F39" t="str">
@@ -13585,7 +13589,7 @@
       <x:c r="D40" t="str">
         <x:v>DEV004</x:v>
       </x:c>
-      <x:c r="E40" t="d">
+      <x:c r="E40" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F40" t="str">
@@ -13608,7 +13612,7 @@
       <x:c r="D41" t="str">
         <x:v>DEV005</x:v>
       </x:c>
-      <x:c r="E41" t="d">
+      <x:c r="E41" s="3" t="d">
         <x:v>2026-10-20T16:00:00.000Z</x:v>
       </x:c>
       <x:c r="F41" t="str">

</xml_diff>